<commit_message>
Re-export the review sheet after the Stage 5 tag changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge_base/review_sheet.xlsx
+++ b/knowledge_base/review_sheet.xlsx
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>patient_education, readmission_context</t>
+          <t>patient_education</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>readmission_context, length_of_stay, discharge_destination</t>
+          <t>readmission_context, length_of_stay</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">

</xml_diff>